<commit_message>
Add the /timeline page: a 3D chrono-spatial view of the names
Depth is time (800-846), places sit on a map of the coast and rivers, Bai Juyi's
postings are a gold thread and each dated name hangs in the year of its poem with
a red arc to where the addressee was. Ends in a side view of the whole span.

- Record sheet: new columns N-Q (year, Bai's place, addressee's post and place),
  read and checked by build.py; Bai's place falls back to content/career.json
- content/places.json (gazetteer), content/career.json (draft postings, unverified)
- public/map/china.json from Natural Earth via tools/fetch_map.py
- Entry pages show the new fields and link to the timeline; nav, About and README updated
- Fixes from the Codex review: overview orientation, closed rings in the map
  simplifier, out-of-span years, mount/unmount race, texture disposal, keyboard
  access, hidden labels catching taps, reduced motion

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/data/Bai-Juyi-Experiment-Record-Sheet.xlsx
+++ b/public/data/Bai-Juyi-Experiment-Record-Sheet.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M36"/>
+  <dimension ref="A1:Q36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -442,6 +442,10 @@
     <col width="11" customWidth="1" min="11" max="11"/>
     <col width="11" customWidth="1" min="12" max="12"/>
     <col width="30" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="18" customWidth="1" min="16" max="16"/>
+    <col width="16" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -508,6 +512,26 @@
       <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Notes / good essay example?</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Year 年 (e.g. 833, 833?, 831-833)</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Bai's place 白居易所在</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Addressee's post 受詩者官職</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Addressee's place 受詩者所在</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record the verdicts for Rounds A and B
Claude Code gave each answer its verdict (columns K and L) by one rule:
an exact match with the person 箋校 names is correct; any other name,
including a name where 箋校 says the name is unknown, is wrong; no name
is "declined", split by whether 箋校 names the person. The site text
now says the verdicts were given by Claude Code, not the student.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/data/Bai-Juyi-Experiment-Record-Sheet.xlsx
+++ b/public/data/Bai-Juyi-Experiment-Record-Sheet.xlsx
@@ -584,8 +584,16 @@
           <t>元稹</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>correct</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>correct</t>
+        </is>
+      </c>
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr">
         <is>
@@ -657,8 +665,16 @@
           <t>劉禹錫</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>correct</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>correct</t>
+        </is>
+      </c>
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr">
         <is>
@@ -730,8 +746,16 @@
           <t>李紳</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>correct</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>correct</t>
+        </is>
+      </c>
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr">
         <is>
@@ -798,8 +822,16 @@
           <t>李紳</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>correct</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>correct</t>
+        </is>
+      </c>
       <c r="M5" t="inlineStr"/>
       <c r="N5" t="inlineStr">
         <is>
@@ -871,8 +903,16 @@
           <t>張籍</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>correct</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>correct</t>
+        </is>
+      </c>
       <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr">
         <is>
@@ -934,8 +974,16 @@
           <t>皇甫曙</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>wrong</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>correct</t>
+        </is>
+      </c>
       <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr">
         <is>
@@ -998,8 +1046,16 @@
           <t>楊汝士</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>correct</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>declined: answer exists</t>
+        </is>
+      </c>
       <c r="M8" t="inlineStr"/>
       <c r="N8" t="inlineStr">
         <is>
@@ -1071,8 +1127,16 @@
           <t>楊汝士</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>correct</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>wrong</t>
+        </is>
+      </c>
       <c r="M9" t="inlineStr"/>
       <c r="N9" t="inlineStr">
         <is>
@@ -1136,8 +1200,16 @@
           <t>楊虞卿</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>declined: answer exists</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>declined: answer exists</t>
+        </is>
+      </c>
       <c r="M10" t="inlineStr"/>
       <c r="N10" t="inlineStr">
         <is>
@@ -1205,8 +1277,16 @@
           <t>（箋校未注受贈人）</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>wrong</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>declined: none exists</t>
+        </is>
+      </c>
       <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr">
         <is>
@@ -1268,8 +1348,16 @@
           <t>牛僧孺</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>correct</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>correct</t>
+        </is>
+      </c>
       <c r="M12" t="inlineStr"/>
       <c r="N12" t="inlineStr">
         <is>
@@ -1337,8 +1425,16 @@
           <t>李宗閔</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>declined: answer exists</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>correct</t>
+        </is>
+      </c>
       <c r="M13" t="inlineStr"/>
       <c r="N13" t="inlineStr">
         <is>
@@ -1410,8 +1506,16 @@
           <t>庾敬休</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>wrong</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>correct</t>
+        </is>
+      </c>
       <c r="M14" t="inlineStr"/>
       <c r="N14" t="inlineStr">
         <is>
@@ -1479,8 +1583,16 @@
           <t>崔韶</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr"/>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>declined: answer exists</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>wrong</t>
+        </is>
+      </c>
       <c r="M15" t="inlineStr"/>
       <c r="N15" t="inlineStr">
         <is>
@@ -1548,8 +1660,16 @@
           <t>韋處厚</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr"/>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>declined: answer exists</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>correct</t>
+        </is>
+      </c>
       <c r="M16" t="inlineStr"/>
       <c r="N16" t="inlineStr">
         <is>
@@ -1621,8 +1741,16 @@
           <t>杜元穎</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr"/>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>correct</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>correct</t>
+        </is>
+      </c>
       <c r="M17" t="inlineStr"/>
       <c r="N17" t="inlineStr">
         <is>
@@ -1694,8 +1822,16 @@
           <t>竇鞏</t>
         </is>
       </c>
-      <c r="K18" t="inlineStr"/>
-      <c r="L18" t="inlineStr"/>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>correct</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>correct</t>
+        </is>
+      </c>
       <c r="M18" t="inlineStr"/>
       <c r="N18" t="inlineStr">
         <is>
@@ -1762,8 +1898,16 @@
           <t>李紳</t>
         </is>
       </c>
-      <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr"/>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>correct</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>correct</t>
+        </is>
+      </c>
       <c r="M19" t="inlineStr"/>
       <c r="N19" t="inlineStr">
         <is>
@@ -1830,8 +1974,16 @@
           <t>獨孤郁</t>
         </is>
       </c>
-      <c r="K20" t="inlineStr"/>
-      <c r="L20" t="inlineStr"/>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>correct</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>correct</t>
+        </is>
+      </c>
       <c r="M20" t="inlineStr"/>
       <c r="N20" t="inlineStr">
         <is>
@@ -1898,8 +2050,16 @@
           <t>嵩陽處士，名未詳（箋：非劉軻）</t>
         </is>
       </c>
-      <c r="K21" t="inlineStr"/>
-      <c r="L21" t="inlineStr"/>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>wrong</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>wrong</t>
+        </is>
+      </c>
       <c r="M21" t="inlineStr"/>
       <c r="N21" t="inlineStr">
         <is>
@@ -1966,8 +2126,16 @@
           <t>舒元輿</t>
         </is>
       </c>
-      <c r="K22" t="inlineStr"/>
-      <c r="L22" t="inlineStr"/>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>correct</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>correct</t>
+        </is>
+      </c>
       <c r="M22" t="inlineStr"/>
       <c r="N22" t="inlineStr">
         <is>
@@ -2030,8 +2198,16 @@
           <t>嚴休復</t>
         </is>
       </c>
-      <c r="K23" t="inlineStr"/>
-      <c r="L23" t="inlineStr"/>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>declined: answer exists</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>correct</t>
+        </is>
+      </c>
       <c r="M23" t="inlineStr"/>
       <c r="N23" t="inlineStr">
         <is>
@@ -2099,8 +2275,16 @@
           <t>崔咸</t>
         </is>
       </c>
-      <c r="K24" t="inlineStr"/>
-      <c r="L24" t="inlineStr"/>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>declined: answer exists</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>wrong</t>
+        </is>
+      </c>
       <c r="M24" t="inlineStr"/>
       <c r="N24" t="inlineStr">
         <is>
@@ -2163,8 +2347,16 @@
           <t>皇甫鏞</t>
         </is>
       </c>
-      <c r="K25" t="inlineStr"/>
-      <c r="L25" t="inlineStr"/>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>wrong</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>declined: answer exists</t>
+        </is>
+      </c>
       <c r="M25" t="inlineStr"/>
       <c r="N25" t="inlineStr">
         <is>
@@ -2231,8 +2423,16 @@
           <t>張仲方</t>
         </is>
       </c>
-      <c r="K26" t="inlineStr"/>
-      <c r="L26" t="inlineStr"/>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>wrong</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>correct</t>
+        </is>
+      </c>
       <c r="M26" t="inlineStr"/>
       <c r="N26" t="inlineStr">
         <is>
@@ -2291,8 +2491,16 @@
           <t>李紳（箋作〔李二十賓客〕，題當讀「李二十／三賓客」）</t>
         </is>
       </c>
-      <c r="K27" t="inlineStr"/>
-      <c r="L27" t="inlineStr"/>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>declined: answer exists</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>declined: answer exists</t>
+        </is>
+      </c>
       <c r="M27" t="inlineStr"/>
       <c r="N27" t="inlineStr">
         <is>
@@ -2351,8 +2559,16 @@
           <t>皇甫湜</t>
         </is>
       </c>
-      <c r="K28" t="inlineStr"/>
-      <c r="L28" t="inlineStr"/>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>declined: answer exists</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>declined: answer exists</t>
+        </is>
+      </c>
       <c r="M28" t="inlineStr"/>
       <c r="N28" t="inlineStr">
         <is>
@@ -2414,8 +2630,16 @@
           <t>吳丹</t>
         </is>
       </c>
-      <c r="K29" t="inlineStr"/>
-      <c r="L29" t="inlineStr"/>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>wrong</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>correct</t>
+        </is>
+      </c>
       <c r="M29" t="inlineStr"/>
       <c r="N29" t="inlineStr">
         <is>
@@ -2477,8 +2701,16 @@
           <t>沈述師（箋疑「四」為「十四」之奪文）</t>
         </is>
       </c>
-      <c r="K30" t="inlineStr"/>
-      <c r="L30" t="inlineStr"/>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>wrong</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>correct</t>
+        </is>
+      </c>
       <c r="M30" t="inlineStr"/>
       <c r="N30" t="inlineStr">
         <is>
@@ -2537,8 +2769,16 @@
           <t>名未詳</t>
         </is>
       </c>
-      <c r="K31" t="inlineStr"/>
-      <c r="L31" t="inlineStr"/>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>declined: none exists</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>declined: none exists</t>
+        </is>
+      </c>
       <c r="M31" t="inlineStr"/>
       <c r="N31" t="inlineStr">
         <is>
@@ -2602,8 +2842,16 @@
           <t>韋縝</t>
         </is>
       </c>
-      <c r="K32" t="inlineStr"/>
-      <c r="L32" t="inlineStr"/>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>declined: answer exists</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>declined: answer exists</t>
+        </is>
+      </c>
       <c r="M32" t="inlineStr"/>
       <c r="N32" t="inlineStr">
         <is>
@@ -2662,8 +2910,16 @@
           <t>白居易同年，名未出（箋：與江州途中詩之李六郎中非一人）</t>
         </is>
       </c>
-      <c r="K33" t="inlineStr"/>
-      <c r="L33" t="inlineStr"/>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>declined: none exists</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>declined: none exists</t>
+        </is>
+      </c>
       <c r="M33" t="inlineStr"/>
       <c r="N33" t="inlineStr">
         <is>
@@ -2730,8 +2986,16 @@
           <t>楊巨源</t>
         </is>
       </c>
-      <c r="K34" t="inlineStr"/>
-      <c r="L34" t="inlineStr"/>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>correct</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>correct</t>
+        </is>
+      </c>
       <c r="M34" t="inlineStr"/>
       <c r="N34" t="inlineStr">
         <is>
@@ -2795,8 +3059,16 @@
           <t>李播</t>
         </is>
       </c>
-      <c r="K35" t="inlineStr"/>
-      <c r="L35" t="inlineStr"/>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>declined: answer exists</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>declined: answer exists</t>
+        </is>
+      </c>
       <c r="M35" t="inlineStr"/>
       <c r="N35" t="inlineStr">
         <is>
@@ -2860,8 +3132,16 @@
           <t>王質夫</t>
         </is>
       </c>
-      <c r="K36" t="inlineStr"/>
-      <c r="L36" t="inlineStr"/>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>declined: answer exists</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>declined: answer exists</t>
+        </is>
+      </c>
       <c r="M36" t="inlineStr"/>
       <c r="N36" t="inlineStr">
         <is>
@@ -2931,11 +3211,11 @@
       </c>
       <c r="B2">
         <f>COUNTIF(Record!K2:K36,"correct")</f>
-        <v/>
+        <v>14</v>
       </c>
       <c r="C2">
         <f>COUNTIF(Record!L2:L36,"correct")</f>
-        <v/>
+        <v>20</v>
       </c>
     </row>
     <row r="3">
@@ -2946,11 +3226,11 @@
       </c>
       <c r="B3">
         <f>COUNTIF(Record!K2:K36,"wrong")</f>
-        <v/>
+        <v>8</v>
       </c>
       <c r="C3">
         <f>COUNTIF(Record!L2:L36,"wrong")</f>
-        <v/>
+        <v>4</v>
       </c>
     </row>
     <row r="4">
@@ -2961,11 +3241,11 @@
       </c>
       <c r="B4">
         <f>COUNTIF(Record!K2:K36,"declined: answer exists")</f>
-        <v/>
+        <v>11</v>
       </c>
       <c r="C4">
         <f>COUNTIF(Record!L2:L36,"declined: answer exists")</f>
-        <v/>
+        <v>8</v>
       </c>
     </row>
     <row r="5">
@@ -2976,11 +3256,11 @@
       </c>
       <c r="B5">
         <f>COUNTIF(Record!K2:K36,"declined: none exists")</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="C5">
         <f>COUNTIF(Record!L2:L36,"declined: none exists")</f>
-        <v/>
+        <v>3</v>
       </c>
     </row>
     <row r="6">
@@ -2991,11 +3271,11 @@
       </c>
       <c r="B6">
         <f>COUNTIF(Record!K2:K36,"partly")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="C6">
         <f>COUNTIF(Record!L2:L36,"partly")</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -3006,11 +3286,11 @@
       </c>
       <c r="B7">
         <f>COUNTA(Record!K2:K36)</f>
-        <v/>
+        <v>35</v>
       </c>
       <c r="C7">
         <f>COUNTA(Record!L2:L36)</f>
-        <v/>
+        <v>35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Show answers 箋校 cannot check as "can't verify", not wrong
- The record sheet gains an evidence status per answer (columns R, S).
  build.py reads it, checks it fits the verdict, and shows a wrong
  answer where 箋校 gives no name (entry 10 A, entry 20 A and B) as a
  new status, "Can't verify 無從核實", with its own colour and icon.
- The Summary tab table keeps the sheet's strict counts, so the check
  against the sheet still matches; a note says how many of the wrong
  answers cannot be checked. Charts and tables count the new status.
- Method explains the strict rule and the evidence status; "Wrong" now
  means only a different person from the one 箋校 names. Entries show
  the evidence status under the verdict.
- run-info.json records the roles (student part still to be filled in).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/data/Bai-Juyi-Experiment-Record-Sheet.xlsx
+++ b/public/data/Bai-Juyi-Experiment-Record-Sheet.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q36"/>
+  <dimension ref="A1:S36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -446,6 +446,7 @@
     <col width="14" customWidth="1" min="15" max="15"/>
     <col width="18" customWidth="1" min="16" max="16"/>
     <col width="16" customWidth="1" min="17" max="17"/>
+    <col width="26" customWidth="1" min="18" max="19"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -534,6 +535,16 @@
           <t>Addressee's place 受詩者所在</t>
         </is>
       </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>A evidence status (vs 箋校)</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>B evidence status (vs 箋校)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -615,6 +626,16 @@
           <t>江陵</t>
         </is>
       </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>matches reference</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>matches reference</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -696,6 +717,16 @@
           <t>汝州</t>
         </is>
       </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>matches reference</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>matches reference</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -772,6 +803,16 @@
           <t>太子賓客分司東都</t>
         </is>
       </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>matches reference</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>matches reference</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -853,6 +894,16 @@
           <t>越州</t>
         </is>
       </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>matches reference</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>matches reference</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -924,6 +975,16 @@
           <t>長安</t>
         </is>
       </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>matches reference</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>matches reference</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -1000,6 +1061,16 @@
           <t>郎中</t>
         </is>
       </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>differs from reference</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>matches reference</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -1077,6 +1148,16 @@
           <t>長安</t>
         </is>
       </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>matches reference</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>declined: answer exists</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -1158,6 +1239,16 @@
           <t>梓州</t>
         </is>
       </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>matches reference</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>differs from reference</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -1231,6 +1322,16 @@
           <t>常州</t>
         </is>
       </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>declined: answer exists</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>declined: answer exists</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -1298,6 +1399,16 @@
           <t>洛陽</t>
         </is>
       </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>unverifiable: not annotated</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>declined: none exists</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -1379,6 +1490,16 @@
           <t>長安</t>
         </is>
       </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>matches reference</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>matches reference</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -1456,6 +1577,16 @@
           <t>長安</t>
         </is>
       </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>declined: answer exists</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>matches reference</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1537,6 +1668,16 @@
           <t>長安</t>
         </is>
       </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>differs from reference</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>matches reference</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1614,6 +1755,16 @@
           <t>果州</t>
         </is>
       </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>declined: answer exists</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>differs from reference</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1691,6 +1842,16 @@
           <t>開州</t>
         </is>
       </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>declined: answer exists</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>matches reference</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1772,6 +1933,16 @@
           <t>長安</t>
         </is>
       </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>matches reference</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>matches reference</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1848,6 +2019,16 @@
           <t>校書郎（箋：是時或已為校書）</t>
         </is>
       </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>matches reference</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>matches reference</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1924,6 +2105,16 @@
           <t>國子助教</t>
         </is>
       </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>matches reference</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>matches reference</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -2000,6 +2191,16 @@
           <t>起居郎</t>
         </is>
       </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>matches reference</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>matches reference</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -2076,6 +2277,16 @@
           <t>處士</t>
         </is>
       </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>unverifiable: name unknown</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>unverifiable: name unknown</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -2152,6 +2363,16 @@
           <t>員外郎（題稱）</t>
         </is>
       </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>matches reference</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>matches reference</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -2229,6 +2450,16 @@
           <t>長安</t>
         </is>
       </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>declined: answer exists</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>matches reference</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -2301,6 +2532,16 @@
           <t>秘書監（右散騎常侍）</t>
         </is>
       </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>declined: answer exists</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>differs from reference</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -2373,6 +2614,16 @@
           <t>太子賓客分司東都</t>
         </is>
       </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>differs from reference</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>declined: answer exists</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -2449,6 +2700,16 @@
           <t>太子賓客分司東都</t>
         </is>
       </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>differs from reference</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>matches reference</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -2517,6 +2778,16 @@
           <t>太子賓客分司東都</t>
         </is>
       </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>declined: answer exists</t>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>declined: answer exists</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -2580,6 +2851,16 @@
           <t>洛陽</t>
         </is>
       </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>declined: answer exists</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>declined: answer exists</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -2651,6 +2932,16 @@
           <t>長安</t>
         </is>
       </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>differs from reference</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>matches reference</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -2727,6 +3018,16 @@
           <t>著作郎</t>
         </is>
       </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>differs from reference</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>matches reference</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -2800,6 +3101,16 @@
           <t>峽州</t>
         </is>
       </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>declined: none exists</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>declined: none exists</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -2868,6 +3179,16 @@
           <t>太子庶子</t>
         </is>
       </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>declined: answer exists</t>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>declined: answer exists</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -2936,6 +3257,16 @@
           <t>郎中</t>
         </is>
       </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>declined: none exists</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>declined: none exists</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -3017,6 +3348,16 @@
           <t>長安</t>
         </is>
       </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>matches reference</t>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>matches reference</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -3090,6 +3431,16 @@
           <t>蘄州</t>
         </is>
       </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>declined: answer exists</t>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>declined: answer exists</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -3158,14 +3509,27 @@
           <t>處士</t>
         </is>
       </c>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>declined: answer exists</t>
+        </is>
+      </c>
+      <c r="S36" t="inlineStr">
+        <is>
+          <t>declined: answer exists</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <dataValidations count="2">
+  <dataValidations count="3">
     <dataValidation sqref="K2:L36" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"correct,wrong,declined: answer exists,declined: none exists,partly"</formula1>
     </dataValidation>
     <dataValidation sqref="E2:E36 G2:G36" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"high,medium,low"</formula1>
+    </dataValidation>
+    <dataValidation sqref="R2:S36" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"matches reference,differs from reference,rejected by reference,unverifiable: not annotated,unverifiable: name unknown,declined: answer exists,declined: none exists"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3178,7 +3542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -3293,6 +3657,150 @@
         <v>35</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Evidence status (Record R, S)</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Condition A (title only)</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Condition B (title + sources)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>matches reference</t>
+        </is>
+      </c>
+      <c r="B10">
+        <f>COUNTIF(Record!R2:R36,"matches reference")</f>
+        <v>14</v>
+      </c>
+      <c r="C10">
+        <f>COUNTIF(Record!S2:S36,"matches reference")</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>differs from reference</t>
+        </is>
+      </c>
+      <c r="B11">
+        <f>COUNTIF(Record!R2:R36,"differs from reference")</f>
+        <v>6</v>
+      </c>
+      <c r="C11">
+        <f>COUNTIF(Record!S2:S36,"differs from reference")</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>rejected by reference</t>
+        </is>
+      </c>
+      <c r="B12">
+        <f>COUNTIF(Record!R2:R36,"rejected by reference")</f>
+        <v>0</v>
+      </c>
+      <c r="C12">
+        <f>COUNTIF(Record!S2:S36,"rejected by reference")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>unverifiable: not annotated</t>
+        </is>
+      </c>
+      <c r="B13">
+        <f>COUNTIF(Record!R2:R36,"unverifiable: not annotated")</f>
+        <v>1</v>
+      </c>
+      <c r="C13">
+        <f>COUNTIF(Record!S2:S36,"unverifiable: not annotated")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>unverifiable: name unknown</t>
+        </is>
+      </c>
+      <c r="B14">
+        <f>COUNTIF(Record!R2:R36,"unverifiable: name unknown")</f>
+        <v>1</v>
+      </c>
+      <c r="C14">
+        <f>COUNTIF(Record!S2:S36,"unverifiable: name unknown")</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>declined: answer exists</t>
+        </is>
+      </c>
+      <c r="B15">
+        <f>COUNTIF(Record!R2:R36,"declined: answer exists")</f>
+        <v>11</v>
+      </c>
+      <c r="C15">
+        <f>COUNTIF(Record!S2:S36,"declined: answer exists")</f>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>declined: none exists</t>
+        </is>
+      </c>
+      <c r="B16">
+        <f>COUNTIF(Record!R2:R36,"declined: none exists")</f>
+        <v>2</v>
+      </c>
+      <c r="C16">
+        <f>COUNTIF(Record!S2:S36,"declined: none exists")</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>total (evidence status)</t>
+        </is>
+      </c>
+      <c r="B17">
+        <f>COUNTA(Record!R2:R36)</f>
+        <v>35</v>
+      </c>
+      <c r="C17">
+        <f>COUNTA(Record!S2:S36)</f>
+        <v>35</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Rows 2-7 keep the original rule: any name 箋校 does not give counts as wrong. Rows 10-17 split those answers by what 箋校 says; nothing is re-judged.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Record the student's own checks of five 箋校 entries; centre the seal text
- run-info.json: the student checked entries 29, 9, 20, 26 and 1 in
  箋校 (30 Oct 2026 HKT) and agreed with all ten verdicts. The record
  sheet's 箋校 reading for entry 29 is corrected (the 「十四」 reading
  is Cen Zhongmian's, which the editor accepts), and entries 26 and 29
  get notes.
- Method: a table of the student's checks under "How answers were
  checked"; the AI-checking limit now says how many entries were
  checked again.
- Seals: the CJK font sets the vertical line and a small bottom
  padding lifts the glyphs, so 樂天 sits centred in the ring.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/data/Bai-Juyi-Experiment-Record-Sheet.xlsx
+++ b/public/data/Bai-Juyi-Experiment-Record-Sheet.xlsx
@@ -2762,7 +2762,11 @@
           <t>declined: answer exists</t>
         </is>
       </c>
-      <c r="M27" t="inlineStr"/>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>Student check (30 Oct 2026): 箋校 reads the title as 李二十／三賓客, so the form of address given to the AI, 李二十三, was itself a misreading. The verdict follows the rule (箋校 names 李紳), but this miss is partly the test's fault.</t>
+        </is>
+      </c>
       <c r="N27" t="inlineStr">
         <is>
           <t>833</t>
@@ -2989,7 +2993,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>沈述師（箋疑「四」為「十四」之奪文）</t>
+          <t>沈述師（箋引岑仲勉《唐人行第錄》，謂「四」係「十四」之奪文，從之）</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -3002,7 +3006,11 @@
           <t>correct</t>
         </is>
       </c>
-      <c r="M30" t="inlineStr"/>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>Student check (30 Oct 2026): the 「十四」 reading is Cen Zhongmian's, which 箋校 accepts (其說是也); column J corrected.</t>
+        </is>
+      </c>
       <c r="N30" t="inlineStr">
         <is>
           <t>837</t>

</xml_diff>